<commit_message>
Sync local non-output changes
</commit_message>
<xml_diff>
--- a/data/MU_conductivity.xlsx
+++ b/data/MU_conductivity.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ssuresh\Projects\report-agent\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://buckmanconnect-my.sharepoint.com/personal/pvenkatesan_buckman_com/Documents/Alarm no.s/Alarm-model/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D022A80D-34DD-4C3E-BD98-48550F04A0AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{D022A80D-34DD-4C3E-BD98-48550F04A0AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9847BB22-17EF-4087-8C1D-F0A23EFF1F13}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E4579A37-90A5-4496-94D4-AFF69FE4F2AD}"/>
   </bookViews>
@@ -1321,7 +1321,7 @@
         <v>37</v>
       </c>
       <c r="D13">
-        <v>8.5</v>
+        <v>300</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1536,7 +1536,7 @@
         <v>79</v>
       </c>
       <c r="D30">
-        <v>2.99</v>
+        <v>300</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -1550,7 +1550,7 @@
         <v>81</v>
       </c>
       <c r="D31">
-        <v>4.68</v>
+        <v>300</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
@@ -1564,7 +1564,7 @@
         <v>83</v>
       </c>
       <c r="D32">
-        <v>5.2</v>
+        <v>300</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -1578,7 +1578,7 @@
         <v>85</v>
       </c>
       <c r="D33">
-        <v>13.53</v>
+        <v>300</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -1592,7 +1592,7 @@
         <v>87</v>
       </c>
       <c r="D34">
-        <v>9.35</v>
+        <v>300</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -1606,7 +1606,7 @@
         <v>89</v>
       </c>
       <c r="D35">
-        <v>4.6900000000000004</v>
+        <v>300</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -1620,7 +1620,7 @@
         <v>91</v>
       </c>
       <c r="D36">
-        <v>4.68</v>
+        <v>300</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -1634,7 +1634,7 @@
         <v>93</v>
       </c>
       <c r="D37">
-        <v>5.84</v>
+        <v>300</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -1648,7 +1648,7 @@
         <v>95</v>
       </c>
       <c r="D38">
-        <v>5.84</v>
+        <v>300</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -1662,7 +1662,7 @@
         <v>97</v>
       </c>
       <c r="D39">
-        <v>13.01</v>
+        <v>300</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
@@ -1676,7 +1676,7 @@
         <v>99</v>
       </c>
       <c r="D40">
-        <v>13.53</v>
+        <v>300</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
@@ -1690,7 +1690,7 @@
         <v>101</v>
       </c>
       <c r="D41">
-        <v>7.73</v>
+        <v>300</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -1704,7 +1704,7 @@
         <v>103</v>
       </c>
       <c r="D42">
-        <v>2.99</v>
+        <v>300</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -1718,7 +1718,7 @@
         <v>105</v>
       </c>
       <c r="D43">
-        <v>11.69</v>
+        <v>300</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
@@ -1732,7 +1732,7 @@
         <v>107</v>
       </c>
       <c r="D44">
-        <v>11.1</v>
+        <v>300</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
@@ -1746,7 +1746,7 @@
         <v>109</v>
       </c>
       <c r="D45">
-        <v>6.08</v>
+        <v>300</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
@@ -1760,7 +1760,7 @@
         <v>111</v>
       </c>
       <c r="D46">
-        <v>5.84</v>
+        <v>300</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
@@ -1774,7 +1774,7 @@
         <v>113</v>
       </c>
       <c r="D47">
-        <v>9.35</v>
+        <v>300</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -1788,7 +1788,7 @@
         <v>115</v>
       </c>
       <c r="D48">
-        <v>11.45</v>
+        <v>300</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
@@ -1802,7 +1802,7 @@
         <v>117</v>
       </c>
       <c r="D49">
-        <v>2.88</v>
+        <v>300</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
@@ -2106,7 +2106,7 @@
         <v>179</v>
       </c>
       <c r="D76">
-        <v>43</v>
+        <v>350</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>